<commit_message>
Wieder auf alte Queue umbenannt
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\korbinian.zacherl\Documents\UiPath\EWO_neu\uipath-rpa_ewo_prod\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C443E413-BE9A-4AA0-8927-5F46CD14CE0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A880BCC3-CDB1-42C6-AEAC-463D89E2BC73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12468" yWindow="13584" windowWidth="17280" windowHeight="8928" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -240,7 +240,7 @@
     <t>javaw</t>
   </si>
   <si>
-    <t>ProcessEWOQueueProd</t>
+    <t>ProcessEWOQueue</t>
   </si>
 </sst>
 </file>

</xml_diff>